<commit_message>
Cập nhật danh mục hàng hóa rủi ro và quy trình xử lý theo Nghị định 37/2026/NĐ-CP & Thông tư 31/2026/TT-BCT
</commit_message>
<xml_diff>
--- a/reports/Danh_sach_Van_ban_Phap_luat_XNK.xlsx
+++ b/reports/Danh_sach_Van_ban_Phap_luat_XNK.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2940,11 +2940,7 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I42" s="2" t="n"/>
       <c r="J42" s="4" t="inlineStr">
         <is>
           <t>Xác định rõ ràng hơn ranh giới và phạm vi hoạt động của cơ quan Hải quan tại khu vực cửa khẩu đường bộ, đường sắt quốc tế, cảng biển và cảng hàng không quốc tế. Quy định chi tiết cơ chế phối hợp tuần tra, kiểm soát và trao đổi thông tin phòng chống buôn lậu giữa Hải quan và Biên phòng, Cảnh sát biển, Công an.</t>
@@ -3000,11 +2996,7 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I43" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I43" s="5" t="n"/>
       <c r="J43" s="7" t="inlineStr">
         <is>
           <t>Cải cách căn bản thủ tục hải quan theo hướng số hóa 100% hồ sơ giấy tờ, lược bỏ các chứng từ không cần thiết. Quy định rõ ràng hơn về thủ tục hải quan đối với hàng hóa xuất nhập khẩu tại chỗ, thắt chặt điều kiện áp dụng chế độ ưu tiên đối với doanh nghiệp logistics.</t>
@@ -3060,11 +3052,7 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I44" s="2" t="n"/>
       <c r="J44" s="4" t="inlineStr">
         <is>
           <t>Điều chỉnh và bổ sung các quy định về miễn thuế, giảm thuế, hoàn thuế xuất nhập khẩu. Đặc biệt bổ sung quy định cụ thể về việc miễn thuế đối với nguyên liệu, vật tư nhập khẩu để sản xuất xuất khẩu và gia công xuất khẩu trong trường hợp có thuê doanh nghiệp khác gia công lại.</t>
@@ -3120,11 +3108,7 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I45" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I45" s="5" t="n"/>
       <c r="J45" s="7" t="inlineStr">
         <is>
           <t>Đơn giản hóa quy trình cấp phép nhập khẩu văn hóa phẩm phi thương mại như sách, báo, tranh ảnh, phim ảnh phục vụ nghiên cứu, hội thảo. Rút ngắn thời gian thẩm định nội dung từ 10 ngày xuống còn 5 ngày làm việc.</t>
@@ -3180,11 +3164,7 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I46" s="2" t="n"/>
       <c r="J46" s="4" t="inlineStr">
         <is>
           <t>Quy định quy trình hải quan điện tử đối với hàng hóa nhóm chuyển phát nhanh (express), đặc biệt là nhóm hàng hóa giao dịch qua các sàn thương mại điện tử xuyên biên giới. Yêu cầu truyền trước thông tin hàng hóa trước khi hàng đến.</t>
@@ -3240,11 +3220,7 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I47" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I47" s="5" t="n"/>
       <c r="J47" s="7" t="inlineStr">
         <is>
           <t>Cập nhật và nội luật hóa các thay đổi mới nhất về Quy tắc xuất xứ hàng hóa (PSR) theo biểu thuế hài hòa toàn cầu mới của Hiệp định AANZFTA nâng cấp. Hướng dẫn chi tiết cách xác định xuất xứ, nộp C/O Form AANZ.</t>
@@ -3300,11 +3276,7 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I48" s="2" t="n"/>
       <c r="J48" s="4" t="inlineStr">
         <is>
           <t>Ban hành hành lang pháp lý toàn diện cho cơ chế tự chứng nhận xuất xứ (Self-Certification) của doanh nghiệp xuất khẩu sang các thị trường có FTA thế hệ mới như CPTPP, EVFTA, RCEP. Quy định điều kiện doanh nghiệp được tự chứng nhận và trách nhiệm hậu kiểm.</t>
@@ -3360,11 +3332,7 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I49" s="5" t="n"/>
       <c r="J49" s="7" t="inlineStr">
         <is>
           <t>Cập nhật danh mục hàng hóa lưỡng dụng (dual-use goods - hàng hóa sử dụng cho cả mục đích dân sự và quân sự) phải có giấy phép nhập khẩu/xuất khẩu chuyên ngành của Bộ Khoa học và Công nghệ. Quy định quy trình kiểm soát chặt chẽ đối với công nghệ và thiết bị nhạy cảm.</t>
@@ -3420,11 +3388,7 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I50" s="2" t="n"/>
       <c r="J50" s="4" t="inlineStr">
         <is>
           <t>Sửa đổi quy trình đăng ký kiểm tra chất lượng nhà nước đối với hàng hóa nhập khẩu nhóm 2 thuộc trách nhiệm quản lý của Bộ BKHCN. Cho phép nộp đăng ký trực tuyến hoàn toàn qua Cổng thông tin một cửa quốc gia (NSW) và thừa nhận kết quả đánh giá hợp chuẩn nước ngoài.</t>
@@ -3480,24 +3444,1764 @@
           <t>Chưa xác định</t>
         </is>
       </c>
-      <c r="I51" s="5" t="inlineStr">
+      <c r="I51" s="5" t="n"/>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>Quy định điều kiện kiểm tra, giám sát chất lượng và cấp chứng thư an toàn thực phẩm (Health Certificate) đối với lô hàng thủy sản xuất khẩu sang các thị trường khó tính (EU, Mỹ, Nhật Bản, Trung Quốc). Quy định rõ quy trình xử lý khi lô hàng xuất khẩu bị cảnh báo ở nước ngoài.</t>
+        </is>
+      </c>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>Hệ thống hóa và siết chặt các tiêu chí kiểm soát hóa chất, kháng sinh cấm trong thủy sản xuất khẩu để đáp ứng các yêu cầu kiểm soát nhập khẩu khắt khe hơn từ phía thị trường nước ngoài.</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="24" customHeight="1">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>117/2026/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Nghị định sửa đổi, bổ sung một số điều của Nghị định số 116/2017/NĐ-CP ngày 17/10/2017 quy định về điều kiện sản xuất, lắp ráp, nhập khẩu và kinh doanh dịch vụ bảo hành, bảo dưỡng ô tô</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Nghị định</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Chính phủ</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>116/2017/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>Nới lỏng một số thủ tục cấp Giấy phép kinh doanh nhập khẩu ô tô và điều kiện bảo hành, bảo dưỡng, tạo cơ hội cho doanh nghiệp nhập khẩu ô tô không chính hãng dễ tiếp cận thị trường hơn, nhưng vẫn duy trì các quy định kỹ thuật nghiêm ngặt để bảo đảm an toàn giao thông và bảo vệ người tiêu dùng.</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>Đơn giản hóa thành phần hồ sơ xin cấp phép nhập khẩu ô tô, giảm thiểu yêu cầu về giấy ủy quyền chính hãng nước ngoài đối với linh kiện phụ tùng thay thế.</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>31/2026/TT-BCT</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Thông tư quy định về truy xuất nguồn gốc sản phẩm, hàng hóa thuộc phạm vi quản lý của Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Thông tư</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="n"/>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>Quy định về quản lý và thực hiện truy xuất nguồn gốc đối với sản phẩm, hàng hóa lưu thông và xuất nhập khẩu thuộc phạm vi quản lý của Bộ Công Thương. Yêu cầu doanh nghiệp thiết lập hệ thống dữ liệu truy xuất và kết nối với Cổng thông tin truy xuất nguồn gốc quốc gia (verigoods.vn).</t>
+        </is>
+      </c>
+      <c r="K53" s="7" t="inlineStr">
+        <is>
+          <t>Chuyển từ cơ chế tự nguyện sang bắt buộc đối với một số nhóm mặt hàng có mức độ rủi ro cao, giúp thắt chặt kiểm soát an toàn và tính minh bạch của hàng hóa.</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="24" customHeight="1">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>22/2026/TT-BNNMT</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Thông tư sửa đổi, bổ sung một số điều quy định về trình tự, thủ tục kiểm dịch thực vật xuất khẩu, nhập khẩu</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Thông tư</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Bộ Nông nghiệp và Môi trường</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>33/2014/TT-BNNPTNT</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>Đơn giản hóa thủ tục hành chính, số hóa hồ sơ kiểm dịch thực vật nhập khẩu, xuất khẩu trên Cổng thông tin một cửa quốc gia, bãi bỏ một số loại giấy tờ bằng giấy không cần thiết nhằm tối ưu hóa hoạt động thông quan hàng nông sản.</t>
+        </is>
+      </c>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>Rút ngắn thời gian xử lý thủ tục cấp giấy chứng nhận kiểm dịch thực vật nhập khẩu/xuất khẩu từ tối đa 24 giờ xuống còn 4 giờ làm việc sau khi kiểm tra đạt yêu cầu.</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>16538/CHQ-NVTHQ</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Công văn hướng dẫn về thủ tục hải quan và thuế GTGT đối với hàng hóa từ nội địa đưa vào doanh nghiệp chế xuất (DNCX)</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="n"/>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t>Hướng dẫn doanh nghiệp nội địa thực hiện thủ tục hải quan tại chỗ khi bán hàng cho doanh nghiệp chế xuất và áp dụng thuế suất thuế GTGT 0% nếu đáp ứng đủ điều kiện về hồ sơ thanh toán không dùng tiền mặt và tờ khai hải quan xuất nhập khẩu tại chỗ.</t>
+        </is>
+      </c>
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t>Làm rõ các vướng mắc kéo dài về thời điểm xuất hóa đơn GTGT điện tử và hồ sơ hải quan đối với các giao dịch mua bán nội địa - chế xuất, tạo sự nhất quán cho các doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="24" customHeight="1">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>14808/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Công văn hướng dẫn thủ tục hải quan đối với hàng hóa đã qua sử dụng đưa vào kho ngoại quan</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>Hướng dẫn chi tiết về việc không cho phép gửi kho ngoại quan đối với các mặt hàng máy móc, thiết bị đã qua sử dụng thuộc danh mục cấm nhập khẩu hoặc tạm ngừng nhập khẩu để bảo vệ môi trường, tránh việc lợi dụng kho ngoại quan để tuồn chất thải công nghiệp vào nội địa.</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>Siết chặt khâu kiểm tra hồ sơ, thông tin xuất xứ và tình trạng thực tế của thiết bị trước khi cho phép bốc dỡ vào kho ngoại quan tại các cảng biển và cửa khẩu.</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="24" customHeight="1">
+      <c r="A57" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>12618/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Công văn giải đáp vướng mắc về thủ tục hải quan đối với hàng hóa cung cấp cho doanh nghiệp chế xuất</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="n"/>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>Hướng dẫn các trường hợp được miễn mở tờ khai hải quan đối với một số nhóm hàng tiêu dùng sinh hoạt hàng ngày (như văn phòng phẩm, lương thực, thực phẩm) đưa từ nội địa vào doanh nghiệp chế xuất phục vụ vận hành văn phòng và đời sống sinh hoạt của nhân viên.</t>
+        </is>
+      </c>
+      <c r="K57" s="7" t="inlineStr">
+        <is>
+          <t>Nới lỏng và đơn giản hóa thủ tục hành chính hải quan đối với giao dịch hàng hóa nhỏ lẻ phục vụ sinh hoạt nội bộ của doanh nghiệp chế xuất, giảm tải khối lượng tờ khai cho chi cục hải quan.</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="24" customHeight="1">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>15395/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Công văn hướng dẫn thủ tục hải quan cho doanh nghiệp ưu tiên trong thời gian hệ thống VNACCS/VCIS tạm dừng bảo trì</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>Hướng dẫn cơ chế cho phép thông quan bằng hồ sơ giấy và thực hiện khai báo bổ sung sau trên hệ thống đối với hàng hóa xuất nhập khẩu của các doanh nghiệp ưu tiên khi hệ thống thông quan điện tử gặp sự cố kỹ thuật lớn hoặc bảo trì định kỳ.</t>
+        </is>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>Bảo đảm hoạt động chuỗi cung ứng không bị gián đoạn, ưu tiên đặc quyền thông quan nhanh cho các đối tượng tuân thủ pháp luật hải quan xuất sắc.</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="24" customHeight="1">
+      <c r="A59" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>8883/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Công văn chỉ đạo các chi cục hải quan ưu tiên thông quan thực phẩm nhập khẩu trong đợt cao điểm Tết Nguyên đán</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="n"/>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>Chỉ đạo triển khai lực lượng trực 24/7, ưu tiên kiểm tra thực tế và thông quan nhanh đối với các lô hàng nông sản, thực phẩm tươi sống nhập khẩu phục vụ nhu cầu thị trường Tết, tránh ách tắc tại cửa khẩu ảnh hưởng đến chất lượng sản phẩm.</t>
+        </is>
+      </c>
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>Biện pháp điều hành hành chính linh hoạt nhằm ổn định cung cầu thị trường tiêu dùng nội địa trong đợt cao điểm mua sắm lớn nhất năm.</t>
+        </is>
+      </c>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="24" customHeight="1">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>54/VBHN-VPQH</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Văn bản hợp nhất Luật Hải quan</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Văn bản hợp nhất</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>Văn phòng Quốc hội</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>54/2014/QH13</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>Văn bản hợp nhất Luật Hải quan 2014 với các nội dung sửa đổi, bổ sung mới nhất từ Luật số 90/2025/QH15 và Luật Công nghệ cao số 133/2025/QH15. Hệ thống lại toàn bộ các quy định pháp lý cao nhất về hải quan tại Việt Nam.</t>
+        </is>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>Cập nhật các thay đổi quan trọng về quyền tự do kinh doanh dịch vụ hải quan, cơ chế quản lý rủi ro và quy trình áp dụng công nghệ cao trong thủ tục thông quan trực tuyến.</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="24" customHeight="1">
+      <c r="A61" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>96/VBHN-VPQH</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Văn bản hợp nhất Luật Thuế xuất khẩu, thuế nhập khẩu</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Văn bản hợp nhất</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Văn phòng Quốc hội</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>107/2016/QH13</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>Văn bản hợp nhất Luật Thuế xuất khẩu, thuế nhập khẩu 2016 với các nội dung được sửa đổi từ các luật thuế mới. Là căn cứ pháp lý cốt lõi để xác định thuế suất ưu đãi, thuế tự vệ và các ưu đãi thuế quan cho doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>Cập nhật các quy định sửa đổi về miễn thuế đối với nguyên liệu nhập khẩu phục vụ nghiên cứu công nghệ cao và hàng hóa phi thương mại, đồng thời chuẩn hóa căn cứ tính thuế.</t>
+        </is>
+      </c>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="24" customHeight="1">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>1075/QĐ-BTC</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Quyết định công bố thủ tục hành chính sửa đổi, bổ sung và bãi bỏ trong lĩnh vực hải quan thuộc phạm vi chức năng quản lý nhà nước của Bộ Tài chính</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Quyết định</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Bộ Tài chính</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="n"/>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>Quyết định công bố việc sửa đổi, bổ sung 07 thủ tục hành chính hải quan và bãi bỏ 12 thủ tục hành chính khác không còn phù hợp, nhằm thúc đẩy chuyển đổi số và tạo điều kiện thông thoáng cho hoạt động xuất nhập khẩu.</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>Cắt giảm 12 thủ tục hành chính trung gian (đăng ký kết nối cổng thông tin tờ khai hải quan điện tử, đăng ký sử dụng chữ ký số một cửa, xác nhận kho xăng dầu đủ điều kiện kiểm tra...). Sửa đổi 07 thủ tục về kho bãi địa điểm làm thủ tục hải quan và hệ thống ACTS.</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="24" customHeight="1">
+      <c r="A63" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>15821/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Công văn về kế hoạch triển khai thí điểm thủ tục hải quan đối với hàng hóa xuất khẩu, nhập khẩu theo mô hình thông quan tập trung</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan - Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="n"/>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>Kế hoạch triển khai thí điểm thủ tục hải quan đối với hàng hóa xuất khẩu, nhập khẩu theo mô hình thông quan tập trung tại Chi cục Hải quan khu vực III. Mục tiêu là tự động hóa các nghiệp vụ hải quan, tạo sự minh bạch và đồng bộ.</t>
+        </is>
+      </c>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>Chuyển từ cơ chế tiếp nhận hồ sơ phi tập trung tại từng chi cục sang tập trung hóa tại địa điểm thí điểm, cho phép luân chuyển và kiểm tra chứng từ qua hệ thống thông tin một cách tự động và đồng bộ hơn.</t>
+        </is>
+      </c>
+      <c r="L63" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="24" customHeight="1">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>15402/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Công văn hướng dẫn về việc nhập khẩu ủy thác cho thương nhân nước ngoài không có hiện diện tại Việt Nam</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan - Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="n"/>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>Hướng dẫn chi tiết về hồ sơ thủ tục và xác định trách nhiệm pháp lý của doanh nghiệp trong nước khi nhận nhập khẩu ủy thác hàng hóa cho đối tác là thương nhân nước ngoài không có hiện diện kinh doanh tại Việt Nam.</t>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>Yêu cầu kiểm soát chặt chẽ hợp đồng ủy thác và định danh rõ vai trò người khai hải quan nhằm tránh tình trạng lợi dụng nhập khẩu ủy thác để trốn thuế hoặc nhập hàng trái quy định.</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="24" customHeight="1">
+      <c r="A65" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>15131/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Công văn trả lời kiến nghị nhập khẩu hàng đã qua sử dụng làm nguyên liệu sản xuất xuất khẩu</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan - Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="n"/>
+      <c r="J65" s="7" t="inlineStr">
+        <is>
+          <t>Hướng dẫn xử lý kiến nghị về nhập khẩu hàng đã qua sử dụng làm nguyên liệu cho sản xuất xuất khẩu (đặc biệt là ngành da giày túi xách). Khẳng định hàng hóa đã qua sử dụng thuộc diện cấm nhập khẩu thì không được nhập khẩu, trừ khi có ý kiến chấp thuận của Bộ quản lý chuyên ngành.</t>
+        </is>
+      </c>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>Làm rõ phạm vi áp dụng của lệnh cấm nhập khẩu hàng tiêu dùng/phế liệu đã qua sử dụng, khẳng định loại hình sản xuất xuất khẩu cũng không nằm ngoài ngoại lệ cấm nhập khẩu nếu không được bộ quản lý phê duyệt.</t>
+        </is>
+      </c>
+      <c r="L65" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="24" customHeight="1">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>15029/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Công văn hướng dẫn thủ tục hải quan đối với người nhập cảnh mang theo vàng trang sức, mỹ nghệ</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan - Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="n"/>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>Hướng dẫn nghiệp vụ kiểm tra và quy định định mức mang vàng trang sức, mỹ nghệ của hành khách nhập cảnh. Định mức từ 300g vàng trở lên bắt buộc phải thực hiện thủ tục khai báo hải quan.</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>Cụ thể hóa quy định khai báo hải quan đối với kim loại quý mang theo người khi xuất nhập cảnh, hỗ trợ công tác chống buôn lậu vàng qua đường hàng không và đường bộ.</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="24" customHeight="1">
+      <c r="A67" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>14196/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Công văn hướng dẫn gia hạn thời gian lưu giữ hàng hóa gửi kho ngoại quan</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan - Tổng cục Hải quan</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="n"/>
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t>Hướng dẫn thủ tục đề xuất gia hạn thời gian lưu giữ hàng hóa tại kho ngoại quan và nghĩa vụ đưa hàng ra khỏi kho khi hết hạn. Quy định quy trình xử lý hàng tồn đọng quá hạn gửi kho ngoại quan.</t>
+        </is>
+      </c>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>Quy định cụ thể các trường hợp bất khả kháng hoặc đứt gãy chuỗi cung ứng được xem xét gia hạn, đồng thời tăng cường giám sát thời gian lưu kho để tránh ách tắc tại các kho ngoại quan lớn.</t>
+        </is>
+      </c>
+      <c r="L67" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="24" customHeight="1">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>02/2026/TT-BCT</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Thông tư quy định một số biện pháp thi hành Luật Hóa chất và Nghị định số 25/2026/NĐ-CP về phát triển ngành công nghiệp hóa chất</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Thông tư</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>32/2017/TT-BCT</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>Quy định quy trình cấp chứng chỉ tư vấn chuyên ngành hóa chất, lập và thẩm định kế hoạch phòng ngừa, ứng phó sự cố hóa chất đối với doanh nghiệp sản xuất, kinh doanh, lưu trữ hóa chất.</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t>Đồng bộ hóa các biểu mẫu và quy trình khai báo hóa chất nhập khẩu phù hợp với Luật Hóa chất sửa đổi, siết chặt các biện pháp đảm bảo an toàn tại kho hóa chất trung chuyển.</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="24" customHeight="1">
+      <c r="A69" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>17/2026/TT-BNNMT</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Thông tư sửa đổi, bổ sung một số điều của Thông tư số 25/2018/TT-BNNPTNT về đánh giá rủi ro và cấp phép nhập khẩu thủy sản sống</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Thông tư</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Bộ Nông nghiệp và Phát triển nông thôn</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>25/2018/TT-BNNPTNT</t>
+        </is>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>Sửa đổi và cập nhật quy trình đánh giá nguy cơ, kiểm dịch sinh học và cấp phép nhập khẩu đối với các loài thủy sản sống đưa vào Việt Nam làm thực phẩm hoặc con giống.</t>
+        </is>
+      </c>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>Rút ngắn thời hạn giải quyết hồ sơ cấp phép nhập khẩu thủy sản sống từ 15 ngày làm việc xuống còn 10 ngày làm việc, đơn giản hóa các biểu mẫu đánh giá rủi ro sinh học.</t>
+        </is>
+      </c>
+      <c r="L69" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="24" customHeight="1">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>165/2026/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Nghị định quy định chi tiết và hướng dẫn thi hành một số điều của Luật Phòng bệnh</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Nghị định</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Chính phủ</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>Quy định chi tiết về tiêm chủng, an toàn sinh học xét nghiệm y tế, quy trình kiểm dịch y tế biên giới đối với người, phương tiện và hàng hóa nhập cảnh, xuất cảnh.</t>
+        </is>
+      </c>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>Cho phép cơ chế mua sắm và đấu thầu khẩn cấp đối với vắc-xin, sinh phẩm y tế nhập khẩu trong các tình huống khẩn cấp, khắc phục vướng mắc về thủ tục nhập khẩu thiết bị y tế công lập.</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="24" customHeight="1">
+      <c r="A71" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>1684/QĐ-BYT</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Quyết định công bố thủ tục hành chính sửa đổi, bổ sung và bãi bỏ trong lĩnh vực phòng bệnh thuộc phạm vi quản lý của Bộ Y tế</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Quyết định</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Bộ Y tế</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="n"/>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
+          <t>Quyết định công bố bãi bỏ 4 thủ tục hành chính và sửa đổi 13 thủ tục hành chính khác nhằm đơn giản hóa điều kiện kinh doanh trong lĩnh vực phòng bệnh (như đăng ký lưu hành chế phẩm diệt côn trùng, diệt khuẩn nhập khẩu).</t>
+        </is>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>Cắt giảm thời gian cấp số đăng ký lưu hành đối với chế phẩm nhập khẩu, tăng cường phân cấp và ủy quyền giải quyết thủ tục hành chính cho Sở Y tế các tỉnh thành.</t>
+        </is>
+      </c>
+      <c r="L71" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="24" customHeight="1">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>1157/QĐ-BCT</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Quyết định 1157/QĐ-BCT về lượng hạn ngạch thuế quan đối với hàng dệt may xuất khẩu sang Mê-hi-cô năm 2026 theo Hiệp định Đối tác Toàn diện và Tiến bộ xuyên Thái Bình Dương (CPTPP)</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Quyết định</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="J51" s="7" t="inlineStr">
-        <is>
-          <t>Quy định điều kiện kiểm tra, giám sát chất lượng và cấp chứng thư an toàn thực phẩm (Health Certificate) đối với lô hàng thủy sản xuất khẩu sang các thị trường khó tính (EU, Mỹ, Nhật Bản, Trung Quốc). Quy định rõ quy trình xử lý khi lô hàng xuất khẩu bị cảnh báo ở nước ngoài.</t>
-        </is>
-      </c>
-      <c r="K51" s="7" t="inlineStr">
-        <is>
-          <t>Hệ thống hóa và siết chặt các tiêu chí kiểm soát hóa chất, kháng sinh cấm trong thủy sản xuất khẩu để đáp ứng các yêu cầu kiểm soát nhập khẩu khắt khe hơn từ phía thị trường nước ngoài.</t>
-        </is>
-      </c>
-      <c r="L51" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>Quy định lượng hạn ngạch thuế quan cụ thể đối với các nhóm hàng dệt may xuất khẩu sang Mexico trong năm 2026 theo Hiệp định CPTPP. Doanh nghiệp cần tuân thủ quy trình đăng ký, kê khai để được phân bổ hạn ngạch hưởng thuế suất ưu đãi đặc biệt.</t>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr">
+        <is>
+          <t>Cụ thể hóa và điều chỉnh hạn ngạch thuế quan xuất khẩu hàng dệt may sang thị trường Mexico cho năm 2026 để phù hợp với lộ trình CPTPP và nhu cầu thực tế của các doanh nghiệp trong nước.</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="24" customHeight="1">
+      <c r="A73" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>1090/QĐ-BCT</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Quyết định 1090/QĐ-BCT về việc công bố thủ tục hành chính mới ban hành trong lĩnh vực xuất nhập khẩu thuộc phạm vi chức năng quản lý của Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Quyết định</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
+          <t>Công bố các thủ tục hành chính mới được thiết lập trong lĩnh vực xuất nhập khẩu, hướng dẫn cụ thể về trình tự thực hiện, cách thức nộp hồ sơ, thành phần hồ sơ và thời hạn giải quyết đối với doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="K73" s="7" t="inlineStr">
+        <is>
+          <t>Bổ sung các thủ tục hành chính mới phát sinh do sự thay đổi của luật hoặc các nghị định mới ban hành gần đây, giúp lấp đầy khoảng trống pháp lý và tạo hành lang pháp lý rõ ràng cho doanh nghiệp thực hiện các giao dịch thương mại quốc tế mới.</t>
+        </is>
+      </c>
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="24" customHeight="1">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>937/QĐ-BCT</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Quyết định 937/QĐ-BCT về việc công bố thủ tục hành chính được sửa đổi, bổ sung trong lĩnh vực xuất nhập khẩu thuộc phạm vi chức năng quản lý của Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Quyết định</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>Sửa đổi, bổ sung một loạt các thủ tục hành chính hiện hành trong lĩnh vực xuất nhập khẩu của Bộ Công Thương nhằm tối ưu hóa quy trình nghiệp vụ.</t>
+        </is>
+      </c>
+      <c r="K74" s="4" t="inlineStr">
+        <is>
+          <t>Cắt giảm một số thành phần hồ sơ trùng lặp, tối giản hóa các biểu mẫu và rút ngắn thời hạn giải quyết đối với một số giấy phép xuất nhập khẩu chuyên ngành so với quy định trước đây.</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="24" customHeight="1">
+      <c r="A75" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>403/QĐ-BCT</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Quyết định 403/QĐ-BCT về việc công bố thủ tục hành chính sửa đổi, bổ sung trong lĩnh vực xuất nhập khẩu thuộc phạm vi chức năng quản lý của Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>Quyết định</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Bộ Công Thương</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>Sửa đổi và bổ sung các thủ tục hành chính liên quan đến cấp Giấy chứng nhận xuất xứ (C/O) và cấp phép xuất nhập khẩu tự động để đáp ứng quá trình điện tử hóa.</t>
+        </is>
+      </c>
+      <c r="K75" s="7" t="inlineStr">
+        <is>
+          <t>Tăng cường liên thông dữ liệu qua Cơ chế một cửa quốc gia, chuyển đổi nhiều thủ tục từ nộp hồ sơ giấy hoặc trực tuyến bán phần sang trực tuyến toàn trình (dịch vụ công trực tuyến mức độ 4) so với quy định cũ.</t>
+        </is>
+      </c>
+      <c r="L75" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="24" customHeight="1">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>16911/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Công văn 16911/CHQ-GSQL hướng dẫn thủ tục nhập khẩu hàng hóa của thương nhân nước ngoài không có hiện diện tại Việt Nam</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>Hướng dẫn chi tiết thủ tục hải quan, quyền lợi và nghĩa vụ thuế của thương nhân nước ngoài không hiện diện tại Việt Nam khi tiến hành nhập khẩu hàng hóa. Làm rõ vai trò của đại lý hải quan và mã số thuế được cấp.</t>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t>Hướng dẫn cụ thể và nhất quán hơn quy trình thực hiện, giúp tháo gỡ vướng mắc về việc đứng tên trên tờ khai và xuất hóa đơn giá trị gia tăng mà các quy định trước đây còn chưa rõ ràng.</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="24" customHeight="1">
+      <c r="A77" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>16873/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Công văn 16873/CHQ-GSQL hướng dẫn thay đổi mục đích sử dụng hàng hóa và tái xuất nguyên liệu nhập khẩu</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>Hướng dẫn doanh nghiệp thủ tục hải quan và hoàn thuế đối với trường hợp nguyên liệu nhập khẩu để sản xuất xuất khẩu nhưng thay đổi mục đích sử dụng chuyển tiêu thụ nội địa hoặc tái xuất trả lại.</t>
+        </is>
+      </c>
+      <c r="K77" s="7" t="inlineStr">
+        <is>
+          <t>Đơn giản hóa quy trình chuyển đổi mục đích sử dụng, không yêu cầu hủy tờ khai ban đầu mà cho phép mở tờ khai mới khai thay đổi mục đích sử dụng, đồng thời làm rõ cách thức xử lý thuế đối với phần nguyên liệu chưa qua chế biến.</t>
+        </is>
+      </c>
+      <c r="L77" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="24" customHeight="1">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>16694/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Công văn 16694/CHQ-GSQL hướng dẫn hoạt động xuất khẩu hàng hóa của doanh nghiệp FDI</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>Quy định rõ ràng về quyền xuất khẩu, nhập khẩu và phân phối của doanh nghiệp FDI. Phân biệt rõ hoạt động sản xuất xuất khẩu và hoạt động thương mại mua hàng nội địa để xuất khẩu để áp dụng đúng chính sách thuế.</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr">
+        <is>
+          <t>Siết chặt việc kê khai thuế GTGT đầu vào và đầu ra đối với hàng hóa thuộc quyền xuất khẩu của doanh nghiệp FDI so với các hướng dẫn trước đó, nhằm ngăn chặn tình trạng trục lợi chính sách ưu đãi dành cho sản xuất xuất khẩu.</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="24" customHeight="1">
+      <c r="A79" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>16535/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Công văn 16535/CHQ-GSQL hướng dẫn thủ tục đối với hàng hóa xuất khẩu chuyển cửa khẩu quá cảnh thay đổi cửa khẩu xuất</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
+        <is>
+          <t>Hướng dẫn thủ tục giám sát hải quan đối với các lô hàng chuyển cửa khẩu kết hợp quá cảnh khi doanh nghiệp thay đổi cửa khẩu xuất thực tế do sự cố giao thông hoặc tắc nghẽn biên giới.</t>
+        </is>
+      </c>
+      <c r="K79" s="7" t="inlineStr">
+        <is>
+          <t>Chuyển từ cơ chế phê duyệt và điều chỉnh thủ công tại chi cục hải quan sang xử lý cập nhật tự động trực tiếp trên hệ thống thông tin hải quan, giúp rút ngắn thời gian ách tắc hàng hóa tại biên giới.</t>
+        </is>
+      </c>
+      <c r="L79" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="24" customHeight="1">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>15662/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Công văn 15662/CHQ-GSQL hướng dẫn vướng mắc ghi nhãn hàng hóa và bảo vệ quyền sở hữu trí tuệ</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>Hướng dẫn xử lý các trường hợp nhãn hàng hóa nhập khẩu không đúng quy định hoặc vi phạm sở hữu trí tuệ, nhãn mác trùng lắp hoặc gây nhầm lẫn về xuất xứ.</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr">
+        <is>
+          <t>Đồng bộ hóa quy trình giám sát nhãn hàng hóa với Nghị định 37/2026/NĐ-CP và Thông tư 06/2026/TT-BTC, thắt chặt việc kiểm tra nhãn gốc tại cửa khẩu trước thông quan so với quy định cũ.</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="24" customHeight="1">
+      <c r="A81" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>14844/CHQ-GSQL</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Công văn 14844/CHQ-GSQL hướng dẫn thủ tục hải quan trong kho ngoại quan và giải quyết làm việc ngoài giờ</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>Công văn</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Cục Giám sát quản lý về Hải quan</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J81" s="7" t="inlineStr">
+        <is>
+          <t>Hướng dẫn thủ tục giám sát hàng hóa ra vào kho ngoại quan và cơ chế phối hợp giải quyết thủ tục thông quan cho doanh nghiệp ngoài giờ làm việc hành chính.</t>
+        </is>
+      </c>
+      <c r="K81" s="7" t="inlineStr">
+        <is>
+          <t>Cho phép đăng ký làm việc ngoài giờ trực tuyến và yêu cầu hệ thống camera giám sát của kho ngoại quan kết nối trực tiếp với Tổng cục Hải quan để giám sát 24/7, thay vì nộp phiếu đề xuất bằng giấy như trước đây.</t>
+        </is>
+      </c>
+      <c r="L81" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>

</xml_diff>